<commit_message>
step 5 reprocess logic
</commit_message>
<xml_diff>
--- a/preprocessorEC/data/change_simulation_map.xlsx
+++ b/preprocessorEC/data/change_simulation_map.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dli2\OneDrive - Montefiore Medicine\Documents\A8 - Contract Atlas\preprocessorEC\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E077614-DB1D-4AE3-B999-42287F3D29AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D9D86DE-DC7C-425E-B288-CDC499715E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35295" yWindow="3840" windowWidth="21600" windowHeight="11400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1845" yWindow="1260" windowWidth="25065" windowHeight="13110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$15</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,17 +28,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="15">
   <si>
     <t>Same Contract</t>
   </si>
   <si>
-    <t>Actual Action_a</t>
-  </si>
-  <si>
-    <t>Actual Action_b</t>
-  </si>
-  <si>
     <t>Create</t>
   </si>
   <si>
@@ -67,6 +61,18 @@
   </si>
   <si>
     <t>Merged</t>
+  </si>
+  <si>
+    <t>Actual Action2_a</t>
+  </si>
+  <si>
+    <t>Actual Action2_b</t>
+  </si>
+  <si>
+    <t>Intended Action</t>
+  </si>
+  <si>
+    <t>Upsert</t>
   </si>
 </sst>
 </file>
@@ -393,258 +399,477 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
     <col min="2" max="2" width="28.7109375" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" customWidth="1"/>
+    <col min="3" max="4" width="25.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>0</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>0</v>
+      </c>
+      <c r="B8" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>0</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>0</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>0</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
         <v>7</v>
       </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>0</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>0</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>0</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>0</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
         <v>8</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>0</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>0</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>1</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
         <v>9</v>
       </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>0</v>
-      </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>0</v>
+      </c>
+      <c r="B21" t="s">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>5</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>0</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" t="s">
+        <v>5</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>1</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2</v>
+      </c>
+      <c r="C23" t="s">
+        <v>2</v>
+      </c>
+      <c r="D23" t="s">
+        <v>5</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>0</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2</v>
+      </c>
+      <c r="C24" t="s">
         <v>7</v>
       </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>4</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>0</v>
-      </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>0</v>
-      </c>
-      <c r="B10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>0</v>
-      </c>
-      <c r="B12" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>0</v>
-      </c>
-      <c r="B13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>1</v>
-      </c>
-      <c r="B14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>1</v>
-      </c>
-      <c r="B15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" t="s">
-        <v>4</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>0</v>
-      </c>
-      <c r="B16" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>1</v>
-      </c>
-      <c r="B17" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17">
+      <c r="D24" t="s">
+        <v>5</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>0</v>
+      </c>
+      <c r="B25" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" t="s">
+        <v>5</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>0</v>
+      </c>
+      <c r="B26" t="s">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" t="s">
+        <v>5</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>0</v>
+      </c>
+      <c r="B27" t="s">
+        <v>2</v>
+      </c>
+      <c r="C27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" t="s">
+        <v>5</v>
+      </c>
+      <c r="E27">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D14" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D14">
-      <sortCondition ref="B2:B14"/>
-      <sortCondition ref="A2:A14"/>
-      <sortCondition ref="C2:C14"/>
+  <autoFilter ref="A1:E15" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E20">
+      <sortCondition ref="B1:B15"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
complete step5 major logics
</commit_message>
<xml_diff>
--- a/preprocessorEC/data/change_simulation_map.xlsx
+++ b/preprocessorEC/data/change_simulation_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dli2\OneDrive - Montefiore Medicine\Documents\A8 - Contract Atlas\preprocessorEC\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D9D86DE-DC7C-425E-B288-CDC499715E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F090D5F2-785F-4913-B798-CC4BFCABF1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1845" yWindow="1260" windowWidth="25065" windowHeight="13110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="29190" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="15">
   <si>
     <t>Same Contract</t>
   </si>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
@@ -864,6 +864,57 @@
       </c>
       <c r="E27">
         <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>0</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>2</v>
+      </c>
+      <c r="D28" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>0</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>0</v>
+      </c>
+      <c r="B30" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bug fix in change simulation + export btn changes for data export
</commit_message>
<xml_diff>
--- a/preprocessorEC/data/change_simulation_map.xlsx
+++ b/preprocessorEC/data/change_simulation_map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dli2\OneDrive - Montefiore Medicine\Documents\A8 - Contract Atlas\preprocessorEC\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F090D5F2-785F-4913-B798-CC4BFCABF1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47A96A15-8B40-4BDE-9551-015187496188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="29190" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="15">
   <si>
     <t>Same Contract</t>
   </si>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
@@ -914,6 +914,23 @@
         <v>14</v>
       </c>
       <c r="E30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>0</v>
+      </c>
+      <c r="B31" t="s">
+        <v>2</v>
+      </c>
+      <c r="C31" t="s">
+        <v>2</v>
+      </c>
+      <c r="D31" t="s">
+        <v>5</v>
+      </c>
+      <c r="E31">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
major changes on change simulation logic to handle mute TP rows and update lookups
</commit_message>
<xml_diff>
--- a/preprocessorEC/data/change_simulation_map.xlsx
+++ b/preprocessorEC/data/change_simulation_map.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dli2\OneDrive - Montefiore Medicine\Documents\A8 - Contract Atlas\preprocessorEC\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47A96A15-8B40-4BDE-9551-015187496188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16870254-5A87-4FE6-9E9C-B20EEC691B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20265" yWindow="3735" windowWidth="29700" windowHeight="13680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$33</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="15">
   <si>
     <t>Same Contract</t>
   </si>
@@ -399,7 +399,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E31"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
@@ -424,7 +425,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -458,7 +459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0</v>
       </c>
@@ -475,7 +476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -492,7 +493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -509,7 +510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0</v>
       </c>
@@ -526,7 +527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>0</v>
       </c>
@@ -543,7 +544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -560,7 +561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -577,7 +578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>0</v>
       </c>
@@ -594,7 +595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>0</v>
       </c>
@@ -611,7 +612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1</v>
       </c>
@@ -628,7 +629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>0</v>
       </c>
@@ -645,7 +646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>0</v>
       </c>
@@ -662,7 +663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>0</v>
       </c>
@@ -679,7 +680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>0</v>
       </c>
@@ -696,7 +697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>0</v>
       </c>
@@ -713,7 +714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>0</v>
       </c>
@@ -730,7 +731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1</v>
       </c>
@@ -747,7 +748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>0</v>
       </c>
@@ -764,7 +765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0</v>
       </c>
@@ -781,7 +782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1</v>
       </c>
@@ -798,7 +799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0</v>
       </c>
@@ -815,7 +816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>0</v>
       </c>
@@ -832,7 +833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>0</v>
       </c>
@@ -849,7 +850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>0</v>
       </c>
@@ -866,7 +867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>0</v>
       </c>
@@ -883,7 +884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>0</v>
       </c>
@@ -900,7 +901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>0</v>
       </c>
@@ -917,7 +918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>0</v>
       </c>
@@ -934,11 +935,64 @@
         <v>1</v>
       </c>
     </row>
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>0</v>
+      </c>
+      <c r="B32" t="s">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2</v>
+      </c>
+      <c r="D32" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>1</v>
+      </c>
+      <c r="B33" t="s">
+        <v>3</v>
+      </c>
+      <c r="C33" t="s">
+        <v>2</v>
+      </c>
+      <c r="D33" t="s">
+        <v>14</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>0</v>
+      </c>
+      <c r="B34" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" t="s">
+        <v>2</v>
+      </c>
+      <c r="D34" t="s">
+        <v>14</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E15" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E20">
-      <sortCondition ref="B1:B15"/>
-    </sortState>
+  <autoFilter ref="A1:E33" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Expire then Create (Create)"/>
+      </filters>
+    </filterColumn>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>